<commit_message>
Add second-pass industries (trucking, construction, property mgmt, realtors, vets), new clusters M and N, refreshed report and data
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011B1eB8CJrPpN9721yrndQJ
</commit_message>
<xml_diff>
--- a/painkiller_workbook.xlsx
+++ b/painkiller_workbook.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V15"/>
+  <dimension ref="A1:V17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -695,43 +695,43 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C Chargeback / processor-hold dispute packaging</t>
+          <t>M Detention / accessorial claim filing for small carriers</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>NEW (added after first pass)</t>
         </is>
       </c>
       <c r="C4" t="n">
         <v>4</v>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>
       </c>
       <c r="F4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J4" t="n">
         <v>2</v>
       </c>
       <c r="K4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M4" t="n">
         <v>3</v>
@@ -743,7 +743,7 @@
         <v>3</v>
       </c>
       <c r="P4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q4" t="n">
         <v>5</v>
@@ -758,7 +758,7 @@
         <v>4</v>
       </c>
       <c r="U4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V4">
         <f>SUM(C4:U4)+H4</f>
@@ -768,7 +768,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>D Lost billable time capture (small law/consulting)</t>
+          <t>C Chargeback / processor-hold dispute packaging</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -777,61 +777,61 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E5" t="n">
         <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G5" t="n">
         <v>4</v>
       </c>
       <c r="H5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I5" t="n">
+        <v>4</v>
+      </c>
+      <c r="J5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K5" t="n">
+        <v>3</v>
+      </c>
+      <c r="L5" t="n">
+        <v>4</v>
+      </c>
+      <c r="M5" t="n">
+        <v>3</v>
+      </c>
+      <c r="N5" t="n">
+        <v>4</v>
+      </c>
+      <c r="O5" t="n">
+        <v>3</v>
+      </c>
+      <c r="P5" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q5" t="n">
         <v>5</v>
       </c>
-      <c r="I5" t="n">
-        <v>2</v>
-      </c>
-      <c r="J5" t="n">
-        <v>4</v>
-      </c>
-      <c r="K5" t="n">
-        <v>5</v>
-      </c>
-      <c r="L5" t="n">
-        <v>3</v>
-      </c>
-      <c r="M5" t="n">
-        <v>3</v>
-      </c>
-      <c r="N5" t="n">
-        <v>4</v>
-      </c>
-      <c r="O5" t="n">
-        <v>4</v>
-      </c>
-      <c r="P5" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>3</v>
-      </c>
       <c r="R5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S5" t="n">
         <v>3</v>
       </c>
       <c r="T5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V5">
         <f>SUM(C5:U5)+H5</f>
@@ -841,7 +841,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>B Overdue-invoice follow-up + lien/notice deadlines (owner-name, not collections)</t>
+          <t>D Lost billable time capture (small law/consulting)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -850,31 +850,31 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4</v>
+      </c>
+      <c r="H6" t="n">
         <v>5</v>
       </c>
-      <c r="E6" t="n">
+      <c r="I6" t="n">
         <v>2</v>
       </c>
-      <c r="F6" t="n">
-        <v>2</v>
-      </c>
-      <c r="G6" t="n">
-        <v>4</v>
-      </c>
-      <c r="H6" t="n">
-        <v>4</v>
-      </c>
-      <c r="I6" t="n">
-        <v>4</v>
-      </c>
       <c r="J6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L6" t="n">
         <v>3</v>
@@ -883,7 +883,7 @@
         <v>3</v>
       </c>
       <c r="N6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O6" t="n">
         <v>4</v>
@@ -895,16 +895,16 @@
         <v>3</v>
       </c>
       <c r="R6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V6">
         <f>SUM(C6:U6)+H6</f>
@@ -914,25 +914,25 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>G Card processing fee audit</t>
+          <t>B Overdue-invoice follow-up + lien/notice deadlines (owner-name, not collections)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>EXISTING #1</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E7" t="n">
         <v>2</v>
       </c>
       <c r="F7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G7" t="n">
         <v>4</v>
@@ -941,37 +941,37 @@
         <v>4</v>
       </c>
       <c r="I7" t="n">
+        <v>4</v>
+      </c>
+      <c r="J7" t="n">
+        <v>3</v>
+      </c>
+      <c r="K7" t="n">
+        <v>4</v>
+      </c>
+      <c r="L7" t="n">
+        <v>3</v>
+      </c>
+      <c r="M7" t="n">
+        <v>3</v>
+      </c>
+      <c r="N7" t="n">
+        <v>3</v>
+      </c>
+      <c r="O7" t="n">
+        <v>4</v>
+      </c>
+      <c r="P7" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>3</v>
+      </c>
+      <c r="R7" t="n">
+        <v>4</v>
+      </c>
+      <c r="S7" t="n">
         <v>2</v>
-      </c>
-      <c r="J7" t="n">
-        <v>3</v>
-      </c>
-      <c r="K7" t="n">
-        <v>4</v>
-      </c>
-      <c r="L7" t="n">
-        <v>3</v>
-      </c>
-      <c r="M7" t="n">
-        <v>3</v>
-      </c>
-      <c r="N7" t="n">
-        <v>5</v>
-      </c>
-      <c r="O7" t="n">
-        <v>3</v>
-      </c>
-      <c r="P7" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>4</v>
-      </c>
-      <c r="R7" t="n">
-        <v>3</v>
-      </c>
-      <c r="S7" t="n">
-        <v>3</v>
       </c>
       <c r="T7" t="n">
         <v>4</v>
@@ -987,28 +987,28 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>L UPS/FedEx late-delivery refunds</t>
+          <t>G Card processing fee audit</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>EXISTING #6</t>
+          <t>EXISTING #1</t>
         </is>
       </c>
       <c r="C8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" t="n">
         <v>2</v>
       </c>
-      <c r="D8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E8" t="n">
-        <v>3</v>
-      </c>
       <c r="F8" t="n">
         <v>4</v>
       </c>
       <c r="G8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H8" t="n">
         <v>4</v>
@@ -1020,10 +1020,10 @@
         <v>3</v>
       </c>
       <c r="K8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M8" t="n">
         <v>3</v>
@@ -1032,13 +1032,13 @@
         <v>5</v>
       </c>
       <c r="O8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P8" t="n">
         <v>4</v>
       </c>
       <c r="Q8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R8" t="n">
         <v>3</v>
@@ -1047,10 +1047,10 @@
         <v>3</v>
       </c>
       <c r="T8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V8">
         <f>SUM(C8:U8)+H8</f>
@@ -1060,28 +1060,28 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>J HVAC manufacturer warranty claim recovery</t>
+          <t>L UPS/FedEx late-delivery refunds</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>EXISTING #4</t>
+          <t>EXISTING #6</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D9" t="n">
         <v>2</v>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
         <v>4</v>
       </c>
       <c r="G9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H9" t="n">
         <v>4</v>
@@ -1093,7 +1093,7 @@
         <v>3</v>
       </c>
       <c r="K9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L9" t="n">
         <v>2</v>
@@ -1102,16 +1102,16 @@
         <v>3</v>
       </c>
       <c r="N9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R9" t="n">
         <v>3</v>
@@ -1120,10 +1120,10 @@
         <v>3</v>
       </c>
       <c r="T9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V9">
         <f>SUM(C9:U9)+H9</f>
@@ -1133,25 +1133,25 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>F Vendor COI / prequal compliance tracking</t>
+          <t>N Unbilled extras / change-order capture (contractors)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>NEW (added after first pass)</t>
         </is>
       </c>
       <c r="C10" t="n">
         <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10" t="n">
         <v>2</v>
       </c>
       <c r="F10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G10" t="n">
         <v>4</v>
@@ -1175,10 +1175,10 @@
         <v>3</v>
       </c>
       <c r="N10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P10" t="n">
         <v>3</v>
@@ -1193,7 +1193,7 @@
         <v>2</v>
       </c>
       <c r="T10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U10" t="n">
         <v>4</v>
@@ -1206,16 +1206,16 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>K Delivery-app dispute recovery</t>
+          <t>J HVAC manufacturer warranty claim recovery</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>EXISTING #5</t>
+          <t>EXISTING #4</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D11" t="n">
         <v>2</v>
@@ -1224,10 +1224,10 @@
         <v>2</v>
       </c>
       <c r="F11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H11" t="n">
         <v>4</v>
@@ -1236,26 +1236,26 @@
         <v>2</v>
       </c>
       <c r="J11" t="n">
+        <v>3</v>
+      </c>
+      <c r="K11" t="n">
+        <v>4</v>
+      </c>
+      <c r="L11" t="n">
         <v>2</v>
       </c>
-      <c r="K11" t="n">
-        <v>3</v>
-      </c>
-      <c r="L11" t="n">
-        <v>3</v>
-      </c>
       <c r="M11" t="n">
+        <v>3</v>
+      </c>
+      <c r="N11" t="n">
+        <v>3</v>
+      </c>
+      <c r="O11" t="n">
+        <v>3</v>
+      </c>
+      <c r="P11" t="n">
         <v>2</v>
       </c>
-      <c r="N11" t="n">
-        <v>4</v>
-      </c>
-      <c r="O11" t="n">
-        <v>3</v>
-      </c>
-      <c r="P11" t="n">
-        <v>3</v>
-      </c>
       <c r="Q11" t="n">
         <v>4</v>
       </c>
@@ -1263,7 +1263,7 @@
         <v>3</v>
       </c>
       <c r="S11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T11" t="n">
         <v>4</v>
@@ -1279,61 +1279,61 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>H Utility bill audit (audit only)</t>
+          <t>F Vendor COI / prequal compliance tracking</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>EXISTING #2</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="C12" t="n">
         <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12" t="n">
         <v>2</v>
       </c>
       <c r="F12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H12" t="n">
         <v>4</v>
       </c>
       <c r="I12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J12" t="n">
         <v>3</v>
       </c>
       <c r="K12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L12" t="n">
+        <v>3</v>
+      </c>
+      <c r="M12" t="n">
+        <v>3</v>
+      </c>
+      <c r="N12" t="n">
         <v>2</v>
       </c>
-      <c r="M12" t="n">
-        <v>3</v>
-      </c>
-      <c r="N12" t="n">
-        <v>5</v>
-      </c>
       <c r="O12" t="n">
+        <v>3</v>
+      </c>
+      <c r="P12" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q12" t="n">
         <v>2</v>
       </c>
-      <c r="P12" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>4</v>
-      </c>
       <c r="R12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S12" t="n">
         <v>2</v>
@@ -1342,7 +1342,7 @@
         <v>4</v>
       </c>
       <c r="U12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V12">
         <f>SUM(C12:U12)+H12</f>
@@ -1352,78 +1352,224 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>I Manufacturer co-op fund recovery</t>
+          <t>K Delivery-app dispute recovery</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>EXISTING #3</t>
+          <t>EXISTING #5</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K13" t="n">
+        <v>3</v>
+      </c>
+      <c r="L13" t="n">
+        <v>3</v>
+      </c>
+      <c r="M13" t="n">
         <v>2</v>
       </c>
-      <c r="L13" t="n">
+      <c r="N13" t="n">
+        <v>4</v>
+      </c>
+      <c r="O13" t="n">
+        <v>3</v>
+      </c>
+      <c r="P13" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>4</v>
+      </c>
+      <c r="R13" t="n">
+        <v>3</v>
+      </c>
+      <c r="S13" t="n">
         <v>2</v>
       </c>
-      <c r="M13" t="n">
-        <v>3</v>
-      </c>
-      <c r="N13" t="n">
-        <v>3</v>
-      </c>
-      <c r="O13" t="n">
-        <v>2</v>
-      </c>
-      <c r="P13" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>4</v>
-      </c>
-      <c r="R13" t="n">
-        <v>3</v>
-      </c>
-      <c r="S13" t="n">
-        <v>3</v>
-      </c>
       <c r="T13" t="n">
         <v>4</v>
       </c>
       <c r="U13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V13">
         <f>SUM(C13:U13)+H13</f>
         <v/>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>H Utility bill audit (audit only)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>EXISTING #2</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4</v>
+      </c>
+      <c r="G14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H14" t="n">
+        <v>4</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" t="n">
+        <v>3</v>
+      </c>
+      <c r="K14" t="n">
+        <v>3</v>
+      </c>
+      <c r="L14" t="n">
+        <v>2</v>
+      </c>
+      <c r="M14" t="n">
+        <v>3</v>
+      </c>
+      <c r="N14" t="n">
+        <v>5</v>
+      </c>
+      <c r="O14" t="n">
+        <v>2</v>
+      </c>
+      <c r="P14" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>4</v>
+      </c>
+      <c r="R14" t="n">
+        <v>2</v>
+      </c>
+      <c r="S14" t="n">
+        <v>2</v>
+      </c>
+      <c r="T14" t="n">
+        <v>4</v>
+      </c>
+      <c r="U14" t="n">
+        <v>3</v>
+      </c>
+      <c r="V14">
+        <f>SUM(C14:U14)+H14</f>
+        <v/>
+      </c>
+    </row>
     <row r="15">
       <c r="A15" t="inlineStr">
+        <is>
+          <t>I Manufacturer co-op fund recovery</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>EXISTING #3</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>4</v>
+      </c>
+      <c r="G15" t="n">
+        <v>3</v>
+      </c>
+      <c r="H15" t="n">
+        <v>3</v>
+      </c>
+      <c r="I15" t="n">
+        <v>1</v>
+      </c>
+      <c r="J15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K15" t="n">
+        <v>2</v>
+      </c>
+      <c r="L15" t="n">
+        <v>2</v>
+      </c>
+      <c r="M15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O15" t="n">
+        <v>2</v>
+      </c>
+      <c r="P15" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>4</v>
+      </c>
+      <c r="R15" t="n">
+        <v>3</v>
+      </c>
+      <c r="S15" t="n">
+        <v>3</v>
+      </c>
+      <c r="T15" t="n">
+        <v>4</v>
+      </c>
+      <c r="U15" t="n">
+        <v>3</v>
+      </c>
+      <c r="V15">
+        <f>SUM(C15:U15)+H15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Criterion 6 (outreach) is counted twice. Scores are my judgment (1-5), not measured. Edit any cell; totals recalc.</t>
         </is>
@@ -1440,7 +1586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -1579,15 +1725,15 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C Chargeback / processor-hold dispute packaging</t>
+          <t>M Detention / accessorial claim filing for small carriers</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1500</v>
+        <v>2400</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ASSUMPTION: $99/mo + share of recovered</t>
+          <t>ASSUMPTION: 5-truck carrier, ~$8k/yr unclaimed detention x 30% fee</t>
         </is>
       </c>
       <c r="D4">
@@ -1595,11 +1741,11 @@
         <v/>
       </c>
       <c r="E4" t="n">
-        <v>150000</v>
+        <v>500000</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>DATA: 2.5-3.5M live Shopify stores; ASSUMPTION 5% big enough to matter</t>
+          <t>UNVERIFIED ASSUMPTION: ~500k small for-hire carriers. WEB: 2.12M total registered carriers (incl. private fleets); ~91.5% run 10 trucks or fewer</t>
         </is>
       </c>
       <c r="G4" s="2">
@@ -1612,22 +1758,22 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>License: none. Obsolescence: medium (Stripe/Shopify shipping native dispute tooling). Margin OK. Purchasing power weak (small merchants).</t>
+          <t>License: none for filing claims in the carrier's name; VERIFY state commercial-collections rules before any escalation. Not brokering. Obsolescence: medium (TMS/ELD vendors and dedicated detention tools already exist). Evidence caveat: several supporting posts look like idea-validation by builders.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>D Lost billable time capture (small law/consulting)</t>
+          <t>C Chargeback / processor-hold dispute packaging</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1188</v>
+        <v>1500</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ASSUMPTION: $99/mo</t>
+          <t>ASSUMPTION: $99/mo + share of recovered</t>
         </is>
       </c>
       <c r="D5">
@@ -1635,11 +1781,11 @@
         <v/>
       </c>
       <c r="E5" t="n">
-        <v>180000</v>
+        <v>150000</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>DATA: ~450k law firms, ~40% solo</t>
+          <t>DATA: 2.5-3.5M live Shopify stores; ASSUMPTION 5% big enough to matter</t>
         </is>
       </c>
       <c r="G5" s="2">
@@ -1652,22 +1798,22 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>FAILS obsolescence: commenters already use AI that logs calls into Clio. Reject.</t>
+          <t>License: none. Obsolescence: medium (Stripe/Shopify shipping native dispute tooling). Margin OK. Purchasing power weak (small merchants).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>B Overdue-invoice follow-up + lien/notice deadlines (owner-name, not collections)</t>
+          <t>D Lost billable time capture (small law/consulting)</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1788</v>
+        <v>1188</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ASSUMPTION: $149/mo done-for-you follow-up</t>
+          <t>ASSUMPTION: $99/mo</t>
         </is>
       </c>
       <c r="D6">
@@ -1675,11 +1821,11 @@
         <v/>
       </c>
       <c r="E6" t="n">
-        <v>1050000</v>
+        <v>180000</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>DATA: ~598k specialty-trade establishments + ~450k law firms (web search)</t>
+          <t>DATA: ~450k law firms, ~40% solo</t>
         </is>
       </c>
       <c r="G6" s="2">
@@ -1692,22 +1838,22 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>License: FAIL if we collect debts for owners; OK only as owner-name reminders/notices. Obsolescence: HIGH (accounting/invoicing software already ships reminders). Margin OK.</t>
+          <t>FAILS obsolescence: commenters already use AI that logs calls into Clio. Reject.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>G Card processing fee audit</t>
+          <t>B Overdue-invoice follow-up + lien/notice deadlines (owner-name, not collections)</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>750</v>
+        <v>1788</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ASSUMPTION: $500k card volume x 0.5% saved x ~30% fee + residual</t>
+          <t>ASSUMPTION: $149/mo done-for-you follow-up</t>
         </is>
       </c>
       <c r="D7">
@@ -1715,11 +1861,11 @@
         <v/>
       </c>
       <c r="E7" t="n">
-        <v>4500000</v>
+        <v>1050000</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>DATA: 6.4M employer firms (SBA); ASSUMPTION ~70% take cards</t>
+          <t>DATA: ~598k specialty-trade establishments + ~450k law firms (web search)</t>
         </is>
       </c>
       <c r="G7" s="2">
@@ -1732,22 +1878,22 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>No license if audit-only; taking processor residuals would be ISO/sales-agent territory (avoid). Many free/contingent audit competitors. Reddit thread shows owners think fees are small next to other costs.</t>
+          <t>License: FAIL if we collect debts for owners; OK only as owner-name reminders/notices. Obsolescence: HIGH (accounting/invoicing software already ships reminders). Margin OK.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>L UPS/FedEx late-delivery refunds</t>
+          <t>G Card processing fee audit</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1500</v>
+        <v>750</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ASSUMPTION: $100k parcel spend x 5% x 30% fee</t>
+          <t>ASSUMPTION: $500k card volume x 0.5% saved x ~30% fee + residual</t>
         </is>
       </c>
       <c r="D8">
@@ -1755,11 +1901,11 @@
         <v/>
       </c>
       <c r="E8" t="n">
-        <v>300000</v>
+        <v>4500000</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>UNVERIFIED: no shipper count found</t>
+          <t>DATA: 6.4M employer firms (SBA); ASSUMPTION ~70% take cards</t>
         </is>
       </c>
       <c r="G8" s="2">
@@ -1772,22 +1918,22 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Real money, but crowded contingency market (25-50% fees) and zero Reddit voice.</t>
+          <t>No license if audit-only; taking processor residuals would be ISO/sales-agent territory (avoid). Many free/contingent audit competitors. Reddit thread shows owners think fees are small next to other costs.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>J HVAC manufacturer warranty claim recovery</t>
+          <t>L UPS/FedEx late-delivery refunds</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ASSUMPTION: $10k recovered x 25% fee</t>
+          <t>ASSUMPTION: $100k parcel spend x 5% x 30% fee</t>
         </is>
       </c>
       <c r="D9">
@@ -1795,11 +1941,11 @@
         <v/>
       </c>
       <c r="E9" t="n">
-        <v>111207</v>
+        <v>300000</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>DATA: 111,207 HVAC/plumbing employer establishments (Census CBP 2023)</t>
+          <t>UNVERIFIED: no shipper count found</t>
         </is>
       </c>
       <c r="G9" s="2">
@@ -1812,14 +1958,14 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Only ~10 relevant posts; one venting HVAC tech. Manufacturer portals differ by brand.</t>
+          <t>Real money, but crowded contingency market (25-50% fees) and zero Reddit voice.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>F Vendor COI / prequal compliance tracking</t>
+          <t>N Unbilled extras / change-order capture (contractors)</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -1852,22 +1998,22 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Low willingness to pay; thin evidence.</t>
+          <t>FAILS obsolescence: contractor software already ships change orders and will add AI capture. Behavior problem (owner freezes), not a tooling gap.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>K Delivery-app dispute recovery</t>
+          <t>J HVAC manufacturer warranty claim recovery</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>750</v>
+        <v>2500</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ASSUMPTION: $3k recoverable x 25% fee</t>
+          <t>ASSUMPTION: $10k recovered x 25% fee</t>
         </is>
       </c>
       <c r="D11">
@@ -1875,11 +2021,11 @@
         <v/>
       </c>
       <c r="E11" t="n">
-        <v>430000</v>
+        <v>111207</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>DATA: ~720k restaurants; ASSUMPTION ~60% on delivery apps</t>
+          <t>DATA: 111,207 HVAC/plumbing employer establishments (Census CBP 2023)</t>
         </is>
       </c>
       <c r="G11" s="2">
@@ -1892,22 +2038,22 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Two relevant complaints; platforms auto-refund customers and give ~10 days to dispute.</t>
+          <t>Only ~10 relevant posts; one venting HVAC tech. Manufacturer portals differ by brand.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>H Utility bill audit (audit only)</t>
+          <t>F Vendor COI / prequal compliance tracking</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>450</v>
+        <v>1188</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ASSUMPTION: $30k utility spend x 5% recovered x 30% fee</t>
+          <t>ASSUMPTION: $99/mo</t>
         </is>
       </c>
       <c r="D12">
@@ -1915,11 +2061,11 @@
         <v/>
       </c>
       <c r="E12" t="n">
-        <v>2000000</v>
+        <v>598000</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>ASSUMPTION: multi-site/high-usage subset of 6.4M employer firms; unverified</t>
+          <t>DATA: ~598k specialty-trade establishments</t>
         </is>
       </c>
       <c r="G12" s="2">
@@ -1932,22 +2078,22 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Almost no Reddit evidence; many established contingency auditors.</t>
+          <t>Low willingness to pay; thin evidence.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>I Manufacturer co-op fund recovery</t>
+          <t>K Delivery-app dispute recovery</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1250</v>
+        <v>750</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ASSUMPTION: $5k claimable x 25% fee</t>
+          <t>ASSUMPTION: $3k recoverable x 25% fee</t>
         </is>
       </c>
       <c r="D13">
@@ -1955,11 +2101,11 @@
         <v/>
       </c>
       <c r="E13" t="n">
-        <v>200000</v>
+        <v>430000</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>WEAK: web says ~43% of small businesses sell national brands; dealer count unverified</t>
+          <t>DATA: ~720k restaurants; ASSUMPTION ~60% on delivery apps</t>
         </is>
       </c>
       <c r="G13" s="2">
@@ -1972,12 +2118,92 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Effectively zero Reddit evidence (one removed MSP post). Manufacturer-by-manufacturer rules kill automation.</t>
+          <t>Two relevant complaints; platforms auto-refund customers and give ~10 days to dispute.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>H Utility bill audit (audit only)</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>450</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ASSUMPTION: $30k utility spend x 5% recovered x 30% fee</t>
+        </is>
+      </c>
+      <c r="D14">
+        <f>ROUNDUP(1000000/B14,0)</f>
+        <v/>
+      </c>
+      <c r="E14" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>ASSUMPTION: multi-site/high-usage subset of 6.4M employer firms; unverified</t>
+        </is>
+      </c>
+      <c r="G14" s="2">
+        <f>D14/E14</f>
+        <v/>
+      </c>
+      <c r="H14">
+        <f>IF(G14&gt;0.03,"RISK","ok")</f>
+        <v/>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Almost no Reddit evidence; many established contingency auditors.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
+        <is>
+          <t>I Manufacturer co-op fund recovery</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1250</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ASSUMPTION: $5k claimable x 25% fee</t>
+        </is>
+      </c>
+      <c r="D15">
+        <f>ROUNDUP(1000000/B15,0)</f>
+        <v/>
+      </c>
+      <c r="E15" t="n">
+        <v>200000</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>WEAK: web says ~43% of small businesses sell national brands; dealer count unverified</t>
+        </is>
+      </c>
+      <c r="G15" s="2">
+        <f>D15/E15</f>
+        <v/>
+      </c>
+      <c r="H15">
+        <f>IF(G15&gt;0.03,"RISK","ok")</f>
+        <v/>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Effectively zero Reddit evidence (one removed MSP post). Manufacturer-by-manufacturer rules kill automation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Blue-sky inputs are ASSUMPTIONS (change column B / E). Market sizes marked DATA came from web searches, not Reddit.</t>
         </is>
@@ -1994,7 +2220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -4329,35 +4555,39 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>J HVAC warranty recovery (existing)</t>
+          <t>M Detention / accessorial claims for small carriers</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>OwnerOperators</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/HVAC/comments/1o2h1lw/</t>
+          <t>https://www.reddit.com/r/OwnerOperators/comments/1rjuuq6/</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>use it with it. Impossible to make a profit recently with all the free warranty labor work from shit products. Carrier, Lennox, Goodman, all</t>
+          <t>went through his logs. 287 hours of detention last year. At $75/hr after free time that's $21,525 just gone. Never filed. That's a used</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>HVAC</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr"/>
+          <t>trucking (8-truck fleet; unverified, low-engagement post)</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>287 hours; $75/hr; $21,525</t>
+        </is>
+      </c>
       <c r="G57" t="n">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="H57" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
@@ -4368,39 +4598,39 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>K Delivery-app disputes (existing)</t>
+          <t>M Detention / accessorial claims for small carriers</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>smallbusiness</t>
+          <t>OwnerOperators</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/smallbusiness/comments/1o72aqi/</t>
+          <t>https://www.reddit.com/r/OwnerOperators/comments/1rdilf4/</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>all small business owners - Uber Eats' "daily ad budget" quietly stacks and double-charges! I paused ads, they still billed me, hid my store,</t>
+          <t>paid their margin. The carrier eats 4 hours of detention because filing is a hassle and the broker knows it. If every carrier filed</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>trucking (owner-operator)</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>$100; $3.88</t>
+          <t>4 hours</t>
         </is>
       </c>
       <c r="G58" t="n">
-        <v>36</v>
+        <v>6</v>
       </c>
       <c r="H58" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
@@ -4411,39 +4641,39 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>K Delivery-app disputes (existing)</t>
+          <t>M Detention / accessorial claims for small carriers</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>smallbusiness</t>
+          <t>OwnerOperators</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/smallbusiness/comments/1sukdal/</t>
+          <t>https://www.reddit.com/r/OwnerOperators/comments/1p3faoc/</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>30% commission). The prices on my page are lower than UberEats because I don't have to inflate them to cover the fees. Problem is</t>
+          <t>Quick Question for O/Os: If ELDs track your truck, why do brokers still deny detention pay? I recently heard that, "While 94.5% of fleets</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>trucking (post may be idea-validation by a builder)</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>5%</t>
         </is>
       </c>
       <c r="G59" t="n">
-        <v>216</v>
+        <v>10</v>
       </c>
       <c r="H59" t="n">
-        <v>164</v>
+        <v>18</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
@@ -4454,37 +4684,808 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
+          <t>M Detention / accessorial claims for small carriers</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Truckers</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/Truckers/comments/1nz38sy/</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>1.5 -2 hours to load you because they won't pay detention pay until after 2 hours my mega loves to tell us daily "we</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>trucking (company driver)</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>2 hours</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>324</v>
+      </c>
+      <c r="H60" t="n">
+        <v>346</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>post</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>M Detention / accessorial claims for small carriers</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Truckers</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/Truckers/comments/1w3uhts/</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>No detention should be illegal Checked in at 9:30am, now 6pm warehouse closed for the day. 8 plus hours of unpaid labor. I love</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>trucking (driver)</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="n">
+        <v>232</v>
+      </c>
+      <c r="H61" t="n">
+        <v>68</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>post</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>M Detention / accessorial claims for small carriers</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Truckers</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/Truckers/comments/1qofr8a/</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>the President, Terry this morning and he's refuses to acknowledge the $1000 in missing payments, including detentions, missing mileage pay and toll reimbursements and</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>trucking (driver vs carrier)</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>$1000</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>513</v>
+      </c>
+      <c r="H62" t="n">
+        <v>76</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>post</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>M Detention / accessorial claims for small carriers</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Truckers</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/Truckers/comments/1v4vfhz/</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>What can I do if broker is refusing to pay layover? I recently picked up a load with "SPI Logistics" from DAT board. I</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>trucking</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>2 days; 5 minutes; $500</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>8</v>
+      </c>
+      <c r="H63" t="n">
+        <v>19</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>post</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>M Detention / accessorial claims for small carriers</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Truckers</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/Truckers/comments/1qj8c52/</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Broker deduction bro got a 500 deduction for missing an appt time by 1 minute and it was due to a long line brokers</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>trucking</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>1 minute</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>28</v>
+      </c>
+      <c r="H64" t="n">
+        <v>37</v>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>post</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>M Detention / accessorial claims for small carriers</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>OwnerOperators</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/OwnerOperators/comments/1p8mk2x/</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>my factoring company sent them the invoice then his company refused to pay the full amount, I asked him what happened he said his</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>trucking (owner-operator vs broker)</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>$750</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>25</v>
+      </c>
+      <c r="H65" t="n">
+        <v>40</v>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>post</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>M Detention / accessorial claims for small carriers</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Truckers</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/Truckers/comments/1q25nof/</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>load. Not so great when you get $17/hr Detention that only starts 2hrs after the appointment time. Not once, not twice, every single pickup</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>trucking (driver)</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>$17/hr</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>72</v>
+      </c>
+      <c r="H66" t="n">
+        <v>63</v>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>post</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>M Detention / accessorial claims for small carriers</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>FreightBrokers</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/FreightBrokers/comments/1qqe635/</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>morning first thing. Carrier is demanding a layover from Tuesday to Wednesday. Is compensation owed to the carrier in this situation?</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>freight brokerage (broker side: claims are judgment calls)</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" t="n">
+        <v>95</v>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>post</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>N Unbilled extras / change orders (contractors)</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/Construction/comments/1qnua1c/</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>+ parts) I realized I gave away about 4 hours a week. At my rate, that is $12,000 a year straight down the drain</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>contracting</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>4 hours; $12,000 a year</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>694</v>
+      </c>
+      <c r="H68" t="n">
+        <v>105</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>post</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>N Unbilled extras / change orders (contractors)</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Contractor</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/Contractor/comments/1u8u7wr/</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>$15,000 with a clear understanding that any additional work would be handled through change orders and paid separately. Today was the first day on</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>contracting</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>$15,000</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>344</v>
+      </c>
+      <c r="H69" t="n">
+        <v>330</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>post</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>N Unbilled extras / change orders (contractors)</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>smallbusiness</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/smallbusiness/comments/1nvziy3/</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>My biggest client asked for a week of free work. I was about to charge them, but deleted the email. I can't risk losing</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>services</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="n">
+        <v>226</v>
+      </c>
+      <c r="H70" t="n">
+        <v>254</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>post</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>M Detention / accessorial claims for small carriers</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>OwnerOperators</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/OwnerOperators/comments/1rjuuq6/_/o8g9h0p/</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>I think most people would pay a fee if you were able to recover this money for them and had hard facts to back</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>trucking (WTP signal, one commenter)</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="n">
+        <v>7</v>
+      </c>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>comment</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>M Detention / accessorial claims for small carriers</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>OwnerOperators</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/OwnerOperators/comments/1r32tpj/_/o51pqv2/</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>it expedited, but at what cost? The minute you file a claim on a brokers bond, they DNU and some even put a freightguard</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>trucking (counter-evidence: retaliation risk)</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="n">
+        <v>8</v>
+      </c>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>comment</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>M Detention / accessorial claims for small carriers</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>OwnerOperators</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/OwnerOperators/comments/1rdilf4/_/o76ubzo/</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>That's because there IS no single answer. Every broker handles it differently, every shipper has different rules, and half the time the rate con</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>trucking (counter-evidence: hard to automate)</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="n">
+        <v>2</v>
+      </c>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>comment</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>M Detention / accessorial claims for small carriers</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>OwnerOperators</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/OwnerOperators/comments/1p3faoc/_/nq4bkbi/</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Brokers pocket it. They'll bill the company but never give carrier an updated rate con. And really there's nothing a carrier can do.</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>trucking</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="n">
+        <v>9</v>
+      </c>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>comment</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>N Unbilled extras / change orders (contractors)</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/Construction/comments/1qnua1c/_/o1whurk/</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Just raise your estimate by a percentage to cover the "good guy tax". That way you save face by not nickel and diming them</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>contracting (counter-evidence: the fix is pricing, not a service)</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="n">
+        <v>569</v>
+      </c>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>comment</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>J HVAC warranty recovery (existing)</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/HVAC/comments/1o2h1lw/</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>use it with it. Impossible to make a profit recently with all the free warranty labor work from shit products. Carrier, Lennox, Goodman, all</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="n">
+        <v>25</v>
+      </c>
+      <c r="H76" t="n">
+        <v>38</v>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>post</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>K Delivery-app disputes (existing)</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>smallbusiness</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/smallbusiness/comments/1o72aqi/</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>all small business owners - Uber Eats' "daily ad budget" quietly stacks and double-charges! I paused ads, they still billed me, hid my store,</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>$100; $3.88</t>
+        </is>
+      </c>
+      <c r="G77" t="n">
+        <v>36</v>
+      </c>
+      <c r="H77" t="n">
+        <v>15</v>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>post</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>K Delivery-app disputes (existing)</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>smallbusiness</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/smallbusiness/comments/1sukdal/</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>30% commission). The prices on my page are lower than UberEats because I don't have to inflate them to cover the fees. Problem is</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="G78" t="n">
+        <v>216</v>
+      </c>
+      <c r="H78" t="n">
+        <v>164</v>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>post</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
           <t>L UPS/FedEx refunds (existing)</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B79" t="inlineStr">
         <is>
           <t>smallbusiness</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C79" t="inlineStr">
         <is>
           <t>https://www.reddit.com/r/smallbusiness/comments/1p68wjj/</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
+      <c r="D79" t="inlineStr">
         <is>
           <t>UPS is charging us heavy surcharges every week. Hi - as the title suggests…I work for a small business and we ship a lot</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr">
+      <c r="E79" t="inlineStr">
         <is>
           <t>small shipper</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="n">
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="n">
         <v>64</v>
       </c>
-      <c r="H60" t="n">
+      <c r="H79" t="n">
         <v>71</v>
       </c>
-      <c r="I60" t="inlineStr">
+      <c r="I79" t="inlineStr">
         <is>
           <t>post</t>
         </is>

</xml_diff>